<commit_message>
Data Description chapter drafted
</commit_message>
<xml_diff>
--- a/results/few_shot_cl_results_fixed.xlsx
+++ b/results/few_shot_cl_results_fixed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/62a6868b0fd06ef7/Desktop/MT_Shashank_CL/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="889" documentId="8_{11DF1DD2-F5A3-42AD-9201-8FAC69274C24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99D6693D-36A7-418F-B627-1252E71A9735}"/>
+  <xr:revisionPtr revIDLastSave="890" documentId="8_{11DF1DD2-F5A3-42AD-9201-8FAC69274C24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{041A4751-8DFF-484D-82DC-10449CFA12EA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0ABF8F8D-A5C6-4B74-9FD9-CAACC9571FF2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{0ABF8F8D-A5C6-4B74-9FD9-CAACC9571FF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="10" r:id="rId1"/>
@@ -746,6 +746,13 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color theme="0"/>
       </font>
@@ -780,13 +787,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <color theme="0"/>
       </font>
@@ -869,12 +869,26 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color theme="0"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -884,21 +898,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -997,7 +997,28 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1007,28 +1028,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1043,6 +1043,20 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color theme="0"/>
       </font>
@@ -1055,20 +1069,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
@@ -1079,7 +1079,14 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1089,7 +1096,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1111,6 +1118,20 @@
       <fill>
         <patternFill>
           <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1137,21 +1158,21 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1161,7 +1182,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1171,28 +1192,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1202,7 +1202,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1212,7 +1212,21 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1243,7 +1257,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1253,7 +1267,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1267,14 +1281,14 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1284,7 +1298,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1294,7 +1308,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1308,6 +1322,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="4" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
@@ -1315,7 +1336,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1325,7 +1346,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1335,28 +1356,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1407,7 +1407,28 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1417,7 +1438,14 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1425,20 +1453,6 @@
       <fill>
         <patternFill>
           <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1448,7 +1462,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1458,7 +1472,28 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1466,20 +1501,6 @@
       <fill>
         <patternFill>
           <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1489,7 +1510,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1499,7 +1520,21 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1507,20 +1542,6 @@
       <fill>
         <patternFill>
           <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1547,21 +1568,14 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1571,7 +1585,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.499984740745262"/>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1581,14 +1595,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1596,13 +1603,6 @@
       <fill>
         <patternFill>
           <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1617,33 +1617,33 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color theme="0"/>
       </font>
       <fill>
         <patternFill>
           <bgColor theme="4" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6637,7 +6637,7 @@
         <v>2.28642136450313E-2</v>
       </c>
       <c r="I92" s="1">
-        <f t="shared" ref="I91:I96" si="22">AVERAGE(C92:H92)</f>
+        <f t="shared" ref="I92:I96" si="22">AVERAGE(C92:H92)</f>
         <v>0.26176491921473288</v>
       </c>
       <c r="J92" s="1"/>
@@ -8714,6 +8714,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A144:M144"/>
+    <mergeCell ref="A100:M100"/>
+    <mergeCell ref="A111:M111"/>
+    <mergeCell ref="A122:M122"/>
+    <mergeCell ref="A133:M133"/>
     <mergeCell ref="A56:M56"/>
     <mergeCell ref="A67:M67"/>
     <mergeCell ref="A78:M78"/>
@@ -8723,28 +8728,23 @@
     <mergeCell ref="A34:M34"/>
     <mergeCell ref="A23:M23"/>
     <mergeCell ref="A45:M45"/>
-    <mergeCell ref="A144:M144"/>
-    <mergeCell ref="A100:M100"/>
-    <mergeCell ref="A111:M111"/>
-    <mergeCell ref="A122:M122"/>
-    <mergeCell ref="A133:M133"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:H9">
-    <cfRule type="cellIs" dxfId="139" priority="66" operator="between">
+    <cfRule type="cellIs" dxfId="139" priority="69" operator="between">
+      <formula>0.6</formula>
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="138" priority="68" operator="between">
+      <formula>0.4</formula>
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="137" priority="67" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="66" operator="between">
       <formula>0.1</formula>
       <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="67" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="137" priority="68" operator="between">
-      <formula>0.4</formula>
-      <formula>0.6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="69" operator="between">
-      <formula>0.6</formula>
-      <formula>0.8</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="135" priority="70" operator="between">
       <formula>0.8</formula>
@@ -8752,69 +8752,69 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:H20">
-    <cfRule type="cellIs" dxfId="134" priority="61" operator="between">
+    <cfRule type="cellIs" dxfId="134" priority="62" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="133" priority="65" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="132" priority="64" operator="between">
+      <formula>0.6</formula>
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="131" priority="63" operator="between">
+      <formula>0.4</formula>
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="130" priority="61" operator="between">
       <formula>0.1</formula>
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="62" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="63" operator="between">
-      <formula>0.4</formula>
-      <formula>0.6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="64" operator="between">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B25:H31">
+    <cfRule type="cellIs" dxfId="129" priority="54" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="65" operator="between">
+    <cfRule type="cellIs" dxfId="128" priority="55" operator="between">
       <formula>0.8</formula>
       <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B25:H31">
-    <cfRule type="cellIs" dxfId="129" priority="51" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="128" priority="52" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="127" priority="53" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="126" priority="54" operator="between">
+    <cfRule type="cellIs" dxfId="126" priority="52" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="125" priority="51" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B36:H42">
+    <cfRule type="cellIs" dxfId="124" priority="60" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="123" priority="59" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="125" priority="55" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B36:H42">
-    <cfRule type="cellIs" dxfId="124" priority="56" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="57" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="122" priority="58" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="59" operator="between">
-      <formula>0.6</formula>
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="60" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
+    <cfRule type="cellIs" dxfId="121" priority="57" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="56" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47:H53">
@@ -8822,43 +8822,43 @@
       <formula>0.1</formula>
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="47" operator="between">
+    <cfRule type="cellIs" dxfId="118" priority="50" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="117" priority="49" operator="between">
+      <formula>0.6</formula>
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="116" priority="48" operator="between">
+      <formula>0.4</formula>
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="47" operator="between">
       <formula>0.2</formula>
       <formula>0.4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="117" priority="48" operator="between">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B58:H64">
+    <cfRule type="cellIs" dxfId="114" priority="45" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="113" priority="43" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="116" priority="49" operator="between">
+    <cfRule type="cellIs" dxfId="112" priority="42" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="111" priority="41" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="110" priority="44" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="50" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B58:H64">
-    <cfRule type="cellIs" dxfId="114" priority="41" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="42" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="43" operator="between">
-      <formula>0.4</formula>
-      <formula>0.6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="44" operator="between">
-      <formula>0.6</formula>
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="45" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69:H75">
@@ -8884,157 +8884,157 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B80:H86">
-    <cfRule type="cellIs" dxfId="104" priority="31" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="32" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
+    <cfRule type="cellIs" dxfId="104" priority="35" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="103" priority="34" operator="between">
+      <formula>0.6</formula>
+      <formula>0.8</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="102" priority="33" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="34" operator="between">
+    <cfRule type="cellIs" dxfId="101" priority="32" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="100" priority="31" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B91:H97">
+    <cfRule type="cellIs" dxfId="99" priority="28" operator="between">
+      <formula>0.4</formula>
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="98" priority="30" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="97" priority="29" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="35" operator="between">
+    <cfRule type="cellIs" dxfId="96" priority="27" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="95" priority="26" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B102:H108">
+    <cfRule type="cellIs" dxfId="94" priority="23" operator="between">
+      <formula>0.4</formula>
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="93" priority="25" operator="between">
       <formula>0.8</formula>
       <formula>1</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B91:H97">
-    <cfRule type="cellIs" dxfId="99" priority="26" operator="between">
+    <cfRule type="cellIs" dxfId="92" priority="24" operator="between">
+      <formula>0.6</formula>
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="91" priority="21" operator="between">
       <formula>0.1</formula>
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="27" operator="between">
+    <cfRule type="cellIs" dxfId="90" priority="22" operator="between">
       <formula>0.2</formula>
       <formula>0.4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="28" operator="between">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B113:H119">
+    <cfRule type="cellIs" dxfId="89" priority="18" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="29" operator="between">
+    <cfRule type="cellIs" dxfId="88" priority="16" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="87" priority="17" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="86" priority="20" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="85" priority="19" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="95" priority="30" operator="between">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B124:H130">
+    <cfRule type="cellIs" dxfId="84" priority="15" operator="between">
       <formula>0.8</formula>
       <formula>1</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B102:H108">
-    <cfRule type="cellIs" dxfId="94" priority="21" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="22" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="23" operator="between">
-      <formula>0.4</formula>
-      <formula>0.6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="24" operator="between">
+    <cfRule type="cellIs" dxfId="83" priority="14" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="25" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B113:H119">
-    <cfRule type="cellIs" dxfId="89" priority="16" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="17" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="87" priority="18" operator="between">
-      <formula>0.4</formula>
-      <formula>0.6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="19" operator="between">
-      <formula>0.6</formula>
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="20" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B124:H130">
-    <cfRule type="cellIs" dxfId="84" priority="11" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="12" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="82" priority="13" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="14" operator="between">
+    <cfRule type="cellIs" dxfId="81" priority="12" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="80" priority="11" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B135:H141">
+    <cfRule type="cellIs" dxfId="79" priority="9" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="15" operator="between">
+    <cfRule type="cellIs" dxfId="78" priority="10" operator="between">
       <formula>0.8</formula>
       <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B135:H141">
-    <cfRule type="cellIs" dxfId="79" priority="6" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="7" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="77" priority="8" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="9" operator="between">
+    <cfRule type="cellIs" dxfId="76" priority="7" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="75" priority="6" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B146:H152">
+    <cfRule type="cellIs" dxfId="74" priority="2" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="73" priority="3" operator="between">
+      <formula>0.4</formula>
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="72" priority="5" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="71" priority="1" operator="between">
+      <formula>0.1</formula>
+      <formula>0.2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="70" priority="4" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="75" priority="10" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B146:H152">
-    <cfRule type="cellIs" dxfId="74" priority="1" operator="between">
-      <formula>0.1</formula>
-      <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="2" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="3" operator="between">
-      <formula>0.4</formula>
-      <formula>0.6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="71" priority="4" operator="between">
-      <formula>0.6</formula>
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="5" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9253,7 +9253,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(C6:H6)</f>
         <v>6.4151048799329831E-4</v>
       </c>
       <c r="J6" s="1"/>
@@ -11558,17 +11558,17 @@
       <formula>0.1</formula>
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="22" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
+    <cfRule type="cellIs" dxfId="68" priority="24" operator="between">
+      <formula>0.6</formula>
+      <formula>0.8</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="67" priority="23" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="24" operator="between">
-      <formula>0.6</formula>
-      <formula>0.8</formula>
+    <cfRule type="cellIs" dxfId="66" priority="22" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="65" priority="25" operator="between">
       <formula>0.8</formula>
@@ -11576,25 +11576,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:H9">
-    <cfRule type="cellIs" dxfId="64" priority="36" operator="between">
+    <cfRule type="cellIs" dxfId="64" priority="40" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="63" priority="36" operator="between">
       <formula>0.1</formula>
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="37" operator="between">
+    <cfRule type="cellIs" dxfId="62" priority="37" operator="between">
       <formula>0.2</formula>
       <formula>0.4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="38" operator="between">
+    <cfRule type="cellIs" dxfId="61" priority="38" operator="between">
       <formula>0.4</formula>
       <formula>0.6</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="39" operator="between">
+    <cfRule type="cellIs" dxfId="60" priority="39" operator="between">
       <formula>0.6</formula>
       <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="40" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:H20">
@@ -11646,21 +11646,21 @@
       <formula>0.1</formula>
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="17" operator="between">
+    <cfRule type="cellIs" dxfId="48" priority="20" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="47" priority="19" operator="between">
+      <formula>0.6</formula>
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="18" operator="between">
+      <formula>0.4</formula>
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="17" operator="between">
       <formula>0.2</formula>
       <formula>0.4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="18" operator="between">
-      <formula>0.4</formula>
-      <formula>0.6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="19" operator="between">
-      <formula>0.6</formula>
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="20" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B53:H59">
@@ -11708,25 +11708,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B75:H81">
-    <cfRule type="cellIs" dxfId="34" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="between">
+      <formula>0.2</formula>
+      <formula>0.4</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="between">
+      <formula>0.4</formula>
+      <formula>0.6</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="4" operator="between">
+      <formula>0.6</formula>
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="5" operator="between">
+      <formula>0.8</formula>
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="1" operator="between">
       <formula>0.1</formula>
       <formula>0.2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="2" operator="between">
-      <formula>0.2</formula>
-      <formula>0.4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="3" operator="between">
-      <formula>0.4</formula>
-      <formula>0.6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="4" operator="between">
-      <formula>0.6</formula>
-      <formula>0.8</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="5" operator="between">
-      <formula>0.8</formula>
-      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>